<commit_message>
update: contest 253 and 254
</commit_message>
<xml_diff>
--- a/CP_Members.xlsx
+++ b/CP_Members.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC contest tracking basic\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FC470F-4A12-43C2-9AD4-022DBA13F62C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="146">
   <si>
     <t>Name</t>
   </si>
@@ -61,402 +55,419 @@
     <t>Starters 252</t>
   </si>
   <si>
+    <t>Starters 253</t>
+  </si>
+  <si>
+    <t>Starters 254</t>
+  </si>
+  <si>
     <t>Ved Mewada</t>
   </si>
   <si>
+    <t>Pratyaksh Rai</t>
+  </si>
+  <si>
+    <t>Manan Singhal</t>
+  </si>
+  <si>
+    <t>MVN AVINASH NAIDU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R. Lenin Fernandez </t>
+  </si>
+  <si>
+    <t>Manisha Bharadwaj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arkajyoti Banerjee </t>
+  </si>
+  <si>
+    <t>Rupayan Roy</t>
+  </si>
+  <si>
+    <t>Shriram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lalam Yasaswi </t>
+  </si>
+  <si>
+    <t>Aayush Talukdar</t>
+  </si>
+  <si>
+    <t>Sudhiksha S</t>
+  </si>
+  <si>
+    <t>Prabjot Singh</t>
+  </si>
+  <si>
+    <t>Akansha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kishor Kumar A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jyoti Yadav </t>
+  </si>
+  <si>
+    <t>B Bhavana Deepthi</t>
+  </si>
+  <si>
+    <t>Joal Yuhanon Thomas</t>
+  </si>
+  <si>
+    <t>Kunj Patel</t>
+  </si>
+  <si>
+    <t>Vishnu Gonuguntla</t>
+  </si>
+  <si>
+    <t>K.G.Dharaneesh</t>
+  </si>
+  <si>
+    <t>anurag rawat</t>
+  </si>
+  <si>
+    <t>M Kavin Velan</t>
+  </si>
+  <si>
+    <t>Rrishabh Sankaran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nookala Kumari Akshara </t>
+  </si>
+  <si>
+    <t>Tanmay Suresh Kotadia</t>
+  </si>
+  <si>
+    <t>Siddharth Silori</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shivsankar S </t>
+  </si>
+  <si>
+    <t>Tanvi Nirmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sudiksha Gupta </t>
+  </si>
+  <si>
+    <t>Abhishek R Iyengar</t>
+  </si>
+  <si>
+    <t>Prince predeep</t>
+  </si>
+  <si>
+    <t>HARITH S R</t>
+  </si>
+  <si>
+    <t>Giridar V.G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aryan Jain </t>
+  </si>
+  <si>
+    <t>U NAREN</t>
+  </si>
+  <si>
+    <t>Subham kumar behera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swati Prasad </t>
+  </si>
+  <si>
+    <t>Sagnik Sen</t>
+  </si>
+  <si>
+    <t>Aswin Bharathi M J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joel Panjimaram Mathew </t>
+  </si>
+  <si>
+    <t>Sankari S</t>
+  </si>
+  <si>
+    <t>Anandha Poorana Thraya S S</t>
+  </si>
+  <si>
     <t>25BCE1969</t>
   </si>
   <si>
+    <t>24BPS1071</t>
+  </si>
+  <si>
+    <t>25BCE1183</t>
+  </si>
+  <si>
+    <t>25BLC1183</t>
+  </si>
+  <si>
+    <t>24BCE1009</t>
+  </si>
+  <si>
+    <t>24BRS1126</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25BEE1216 </t>
+  </si>
+  <si>
+    <t>24BAI1229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25BAI1619 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">24BAI1204 </t>
+  </si>
+  <si>
+    <t>25BCE5826</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24BAI1313 </t>
+  </si>
+  <si>
+    <t>25BCE5163</t>
+  </si>
+  <si>
+    <t>25BCE5532</t>
+  </si>
+  <si>
+    <t>25BCE5811</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24BAI1639 </t>
+  </si>
+  <si>
+    <t>23BRS1170</t>
+  </si>
+  <si>
+    <t>25BEC1033</t>
+  </si>
+  <si>
+    <t>25BCE5591</t>
+  </si>
+  <si>
+    <t>25BCE5054</t>
+  </si>
+  <si>
+    <t>25BCE5063</t>
+  </si>
+  <si>
+    <t>25brs1128</t>
+  </si>
+  <si>
+    <t>25MID1016</t>
+  </si>
+  <si>
+    <t>24BAI1071</t>
+  </si>
+  <si>
+    <t>25brs1111</t>
+  </si>
+  <si>
+    <t>24BCE5281</t>
+  </si>
+  <si>
+    <t>25BAI1368</t>
+  </si>
+  <si>
+    <t>25BCE1735</t>
+  </si>
+  <si>
+    <t>25BCE1336</t>
+  </si>
+  <si>
+    <t>25BCE1824</t>
+  </si>
+  <si>
+    <t>24MIA1042</t>
+  </si>
+  <si>
+    <t>24MIS1007</t>
+  </si>
+  <si>
+    <t>25BCE5179</t>
+  </si>
+  <si>
+    <t>25BCE5162</t>
+  </si>
+  <si>
+    <t>25bce1910</t>
+  </si>
+  <si>
+    <t>25BDS1181</t>
+  </si>
+  <si>
+    <t>24BCE5322</t>
+  </si>
+  <si>
+    <t>25BCE5589</t>
+  </si>
+  <si>
+    <t>24BCE5309</t>
+  </si>
+  <si>
+    <t>24MIS1080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24BAI1426 </t>
+  </si>
+  <si>
+    <t>24MIS1079</t>
+  </si>
+  <si>
+    <t>25BCE1143</t>
+  </si>
+  <si>
     <t>ved1969</t>
   </si>
   <si>
+    <t>pratyakshrai01</t>
+  </si>
+  <si>
+    <t>Entity_404</t>
+  </si>
+  <si>
+    <t>Avinash95512</t>
+  </si>
+  <si>
+    <t>grand_glow_31</t>
+  </si>
+  <si>
+    <t>manisha_14star</t>
+  </si>
+  <si>
+    <t>cheer_atom_78</t>
+  </si>
+  <si>
+    <t>most_fury_06</t>
+  </si>
+  <si>
+    <t>nooblypro</t>
+  </si>
+  <si>
+    <t>scurry_feat_49</t>
+  </si>
+  <si>
+    <t>aayush_dev2101</t>
+  </si>
+  <si>
+    <t>giddy_pine_36</t>
+  </si>
+  <si>
+    <t>prabjot_singh</t>
+  </si>
+  <si>
+    <t>gaze_98</t>
+  </si>
+  <si>
+    <t>kishorkumar007</t>
+  </si>
+  <si>
+    <t>jyotiyadav24</t>
+  </si>
+  <si>
+    <t>bhavana2023</t>
+  </si>
+  <si>
+    <t>joalyt</t>
+  </si>
+  <si>
+    <t>kunj_008</t>
+  </si>
+  <si>
+    <t>mainvishnuhoon</t>
+  </si>
+  <si>
+    <t>headboy14</t>
+  </si>
+  <si>
+    <t>anuragggg</t>
+  </si>
+  <si>
+    <t>kavin2007</t>
+  </si>
+  <si>
+    <t>knot_treat_60</t>
+  </si>
+  <si>
+    <t>ind_akshara</t>
+  </si>
+  <si>
+    <t>tanmaykotadia</t>
+  </si>
+  <si>
+    <t>Siddycodes_101</t>
+  </si>
+  <si>
+    <t>sshivsankar19</t>
+  </si>
+  <si>
+    <t>tan_v_25</t>
+  </si>
+  <si>
+    <t>pure_seed_53</t>
+  </si>
+  <si>
+    <t>abhishek121206</t>
+  </si>
+  <si>
+    <t>harithsr</t>
+  </si>
+  <si>
+    <t>giridar_2007</t>
+  </si>
+  <si>
+    <t>aryanvjain20</t>
+  </si>
+  <si>
+    <t>naren_dev24k</t>
+  </si>
+  <si>
+    <t>biswa_pra_05</t>
+  </si>
+  <si>
+    <t>swatiprasad_26</t>
+  </si>
+  <si>
+    <t>sagnik_sen</t>
+  </si>
+  <si>
+    <t>calm_foxes_49</t>
+  </si>
+  <si>
+    <t>worm_luck_27</t>
+  </si>
+  <si>
+    <t>varsh_2025</t>
+  </si>
+  <si>
+    <t>apt_code_1903</t>
+  </si>
+  <si>
     <t>Core</t>
   </si>
   <si>
+    <t>Present</t>
+  </si>
+  <si>
     <t>Absent</t>
-  </si>
-  <si>
-    <t>Pratyaksh Rai</t>
-  </si>
-  <si>
-    <t>24BPS1071</t>
-  </si>
-  <si>
-    <t>pratyakshrai01</t>
-  </si>
-  <si>
-    <t>Manan Singhal</t>
-  </si>
-  <si>
-    <t>25BCE1183</t>
-  </si>
-  <si>
-    <t>Entity_404</t>
-  </si>
-  <si>
-    <t>MVN AVINASH NAIDU</t>
-  </si>
-  <si>
-    <t>25BLC1183</t>
-  </si>
-  <si>
-    <t>Avinash95512</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R. Lenin Fernandez </t>
-  </si>
-  <si>
-    <t>24BCE1009</t>
-  </si>
-  <si>
-    <t>grand_glow_31</t>
-  </si>
-  <si>
-    <t>Manisha Bharadwaj</t>
-  </si>
-  <si>
-    <t>24BRS1126</t>
-  </si>
-  <si>
-    <t>manisha_14star</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arkajyoti Banerjee </t>
-  </si>
-  <si>
-    <t xml:space="preserve">25BEE1216 </t>
-  </si>
-  <si>
-    <t>cheer_atom_78</t>
-  </si>
-  <si>
-    <t>Rupayan Roy</t>
-  </si>
-  <si>
-    <t>24BAI1229</t>
-  </si>
-  <si>
-    <t>most_fury_06</t>
-  </si>
-  <si>
-    <t>Shriram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25BAI1619 </t>
-  </si>
-  <si>
-    <t>nooblypro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lalam Yasaswi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">24BAI1204 </t>
-  </si>
-  <si>
-    <t>scurry_feat_49</t>
-  </si>
-  <si>
-    <t>Aayush Talukdar</t>
-  </si>
-  <si>
-    <t>25BCE5826</t>
-  </si>
-  <si>
-    <t>aayush_dev2101</t>
-  </si>
-  <si>
-    <t>Sudhiksha S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24BAI1313 </t>
-  </si>
-  <si>
-    <t>giddy_pine_36</t>
-  </si>
-  <si>
-    <t>Prabjot Singh</t>
-  </si>
-  <si>
-    <t>25BCE5163</t>
-  </si>
-  <si>
-    <t>prabjot_singh</t>
-  </si>
-  <si>
-    <t>Akansha</t>
-  </si>
-  <si>
-    <t>25BCE5532</t>
-  </si>
-  <si>
-    <t>gaze_98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kishor Kumar A </t>
-  </si>
-  <si>
-    <t>25BCE5811</t>
-  </si>
-  <si>
-    <t>kishorkumar007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jyoti Yadav </t>
-  </si>
-  <si>
-    <t xml:space="preserve">24BAI1639 </t>
-  </si>
-  <si>
-    <t>jyotiyadav24</t>
-  </si>
-  <si>
-    <t>B Bhavana Deepthi</t>
-  </si>
-  <si>
-    <t>23BRS1170</t>
-  </si>
-  <si>
-    <t>bhavana2023</t>
-  </si>
-  <si>
-    <t>Joal Yuhanon Thomas</t>
-  </si>
-  <si>
-    <t>25BEC1033</t>
-  </si>
-  <si>
-    <t>joalyt</t>
-  </si>
-  <si>
-    <t>Kunj Patel</t>
-  </si>
-  <si>
-    <t>25BCE5591</t>
-  </si>
-  <si>
-    <t>kunj_008</t>
-  </si>
-  <si>
-    <t>Vishnu Gonuguntla</t>
-  </si>
-  <si>
-    <t>25BCE5054</t>
-  </si>
-  <si>
-    <t>mainvishnuhoon</t>
-  </si>
-  <si>
-    <t>K.G.Dharaneesh</t>
-  </si>
-  <si>
-    <t>25BCE5063</t>
-  </si>
-  <si>
-    <t>headboy14</t>
-  </si>
-  <si>
-    <t>anurag rawat</t>
-  </si>
-  <si>
-    <t>25brs1128</t>
-  </si>
-  <si>
-    <t>anuragggg</t>
-  </si>
-  <si>
-    <t>M Kavin Velan</t>
-  </si>
-  <si>
-    <t>25MID1016</t>
-  </si>
-  <si>
-    <t>kavin2007</t>
-  </si>
-  <si>
-    <t>Rrishabh Sankaran</t>
-  </si>
-  <si>
-    <t>24BAI1071</t>
-  </si>
-  <si>
-    <t>knot_treat_60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nookala Kumari Akshara </t>
-  </si>
-  <si>
-    <t>25brs1111</t>
-  </si>
-  <si>
-    <t>ind_akshara</t>
-  </si>
-  <si>
-    <t>Tanmay Suresh Kotadia</t>
-  </si>
-  <si>
-    <t>24BCE5281</t>
-  </si>
-  <si>
-    <t>tanmaykotadia</t>
-  </si>
-  <si>
-    <t>Siddharth Silori</t>
-  </si>
-  <si>
-    <t>25BAI1368</t>
-  </si>
-  <si>
-    <t>Siddycodes_101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shivsankar S </t>
-  </si>
-  <si>
-    <t>25BCE1735</t>
-  </si>
-  <si>
-    <t>sshivsankar19</t>
-  </si>
-  <si>
-    <t>Tanvi Nirmal</t>
-  </si>
-  <si>
-    <t>25BCE1336</t>
-  </si>
-  <si>
-    <t>tan_v_25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sudiksha Gupta </t>
-  </si>
-  <si>
-    <t>25BCE1824</t>
-  </si>
-  <si>
-    <t>pure_seed_53</t>
-  </si>
-  <si>
-    <t>Abhishek R Iyengar</t>
-  </si>
-  <si>
-    <t>24MIA1042</t>
-  </si>
-  <si>
-    <t>abhishek121206</t>
-  </si>
-  <si>
-    <t>Prince predeep</t>
-  </si>
-  <si>
-    <t>24MIS1007</t>
-  </si>
-  <si>
-    <t>HARITH S R</t>
-  </si>
-  <si>
-    <t>25BCE5179</t>
-  </si>
-  <si>
-    <t>harithsr</t>
-  </si>
-  <si>
-    <t>Giridar V.G</t>
-  </si>
-  <si>
-    <t>25BCE5162</t>
-  </si>
-  <si>
-    <t>giridar_2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aryan Jain </t>
-  </si>
-  <si>
-    <t>25bce1910</t>
-  </si>
-  <si>
-    <t>aryanvjain20</t>
-  </si>
-  <si>
-    <t>U NAREN</t>
-  </si>
-  <si>
-    <t>25BDS1181</t>
-  </si>
-  <si>
-    <t>naren_dev24k</t>
-  </si>
-  <si>
-    <t>Subham kumar behera</t>
-  </si>
-  <si>
-    <t>24BCE5322</t>
-  </si>
-  <si>
-    <t>biswa_pra_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swati Prasad </t>
-  </si>
-  <si>
-    <t>25BCE5589</t>
-  </si>
-  <si>
-    <t>swatiprasad_26</t>
-  </si>
-  <si>
-    <t>Sagnik Sen</t>
-  </si>
-  <si>
-    <t>24BCE5309</t>
-  </si>
-  <si>
-    <t>sagnik_sen</t>
-  </si>
-  <si>
-    <t>Aswin Bharathi M J</t>
-  </si>
-  <si>
-    <t>24MIS1080</t>
-  </si>
-  <si>
-    <t>calm_foxes_49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joel Panjimaram Mathew </t>
-  </si>
-  <si>
-    <t xml:space="preserve">24BAI1426 </t>
-  </si>
-  <si>
-    <t>worm_luck_27</t>
-  </si>
-  <si>
-    <t>Sankari S</t>
-  </si>
-  <si>
-    <t>24MIS1079</t>
-  </si>
-  <si>
-    <t>varsh_2025</t>
-  </si>
-  <si>
-    <t>Anandha Poorana Thraya S S</t>
-  </si>
-  <si>
-    <t>25BCE1143</t>
-  </si>
-  <si>
-    <t>apt_code_1903</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -472,7 +483,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -480,26 +491,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -787,116 +808,128 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M45"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="C2">
         <v>9998667888</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
+        <v>143</v>
+      </c>
+      <c r="H2" t="s">
+        <v>144</v>
+      </c>
+      <c r="I2">
+        <v>13</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2">
-        <v>11</v>
-      </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-      <c r="K2">
-        <v>4</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="C3">
         <v>8467095435</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I3">
         <v>5</v>
@@ -913,31 +946,37 @@
       <c r="M3">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>7357511041</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H4" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I4">
         <v>11</v>
@@ -954,31 +993,37 @@
       <c r="M4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="C5">
         <v>9177202100</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I5">
         <v>7</v>
@@ -995,37 +1040,43 @@
       <c r="M5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C6">
         <v>7395927689</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H6" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>2</v>
@@ -1036,31 +1087,37 @@
       <c r="M6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>7870068838</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H7" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1077,37 +1134,43 @@
       <c r="M7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="C8">
         <v>8240087955</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="G8" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H8" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I8">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8">
         <v>4</v>
@@ -1118,31 +1181,37 @@
       <c r="M8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="C9">
         <v>7603913238</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>108</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>38</v>
+        <v>108</v>
       </c>
       <c r="G9" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H9" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1159,37 +1228,43 @@
       <c r="M9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="C10">
         <v>9884464562</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H10" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I10">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10">
         <v>3</v>
@@ -1200,31 +1275,37 @@
       <c r="M10">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="C11">
         <v>9030730696</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>110</v>
       </c>
       <c r="G11" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H11" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I11">
         <v>10</v>
@@ -1241,37 +1322,43 @@
       <c r="M11">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="C12">
         <v>6372111245</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="G12" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H12" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I12">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12">
         <v>4</v>
@@ -1282,31 +1369,37 @@
       <c r="M12">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>7386723779</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="G13" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H13" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I13">
         <v>6</v>
@@ -1323,37 +1416,43 @@
       <c r="M13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>7006933519</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E14" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="G14" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H14" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I14">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14">
         <v>4</v>
@@ -1364,31 +1463,37 @@
       <c r="M14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>9935712711</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H15" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I15">
         <v>6</v>
@@ -1405,31 +1510,37 @@
       <c r="M15">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C16">
         <v>9003223034</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="E16" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F16" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="G16" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H16" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I16">
         <v>4</v>
@@ -1446,37 +1557,43 @@
       <c r="M16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C17">
         <v>8950799910</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="F17" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="G17" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H17" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -1487,31 +1604,37 @@
       <c r="M17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>9398172990</v>
       </c>
       <c r="D18" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="E18" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="F18" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="G18" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H18" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I18">
         <v>2</v>
@@ -1528,37 +1651,43 @@
       <c r="M18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C19">
         <v>9895297289</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H19" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K19">
         <v>1</v>
@@ -1569,37 +1698,43 @@
       <c r="M19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C20">
         <v>9399234486</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H20" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I20">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K20">
         <v>3</v>
@@ -1610,37 +1745,43 @@
       <c r="M20">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C21">
         <v>8390904936</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="G21" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I21">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21">
         <v>3</v>
@@ -1651,31 +1792,37 @@
       <c r="M21">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C22">
         <v>9025580044</v>
       </c>
       <c r="D22" t="s">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="E22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="G22" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H22" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I22">
         <v>12</v>
@@ -1692,10 +1839,16 @@
       <c r="M22">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="B23" t="s">
         <v>79</v>
@@ -1704,60 +1857,66 @@
         <v>8718946895</v>
       </c>
       <c r="D23" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
         <v>79</v>
       </c>
       <c r="F23" t="s">
+        <v>122</v>
+      </c>
+      <c r="G23" t="s">
+        <v>143</v>
+      </c>
+      <c r="H23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" t="s">
         <v>80</v>
-      </c>
-      <c r="G23" t="s">
-        <v>16</v>
-      </c>
-      <c r="H23" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" t="s">
-        <v>82</v>
       </c>
       <c r="C24">
         <v>7305542772</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="E24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F24" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="G24" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H24" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -1774,37 +1933,43 @@
       <c r="M24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C25">
         <v>9655635923</v>
       </c>
       <c r="D25" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="E25" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F25" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="G25" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H25" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I25">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K25">
         <v>4</v>
@@ -1815,37 +1980,43 @@
       <c r="M25">
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C26">
         <v>6301777824</v>
       </c>
       <c r="D26" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="E26" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="F26" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="G26" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H26" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I26">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K26">
         <v>4</v>
@@ -1856,31 +2027,37 @@
       <c r="M26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C27">
         <v>956211707</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>126</v>
       </c>
       <c r="E27" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F27" t="s">
-        <v>92</v>
+        <v>126</v>
       </c>
       <c r="G27" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H27" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I27">
         <v>3</v>
@@ -1897,31 +2074,37 @@
       <c r="M27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C28">
         <v>7017097553</v>
       </c>
       <c r="D28" t="s">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="E28" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="F28" t="s">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="G28" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H28" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I28">
         <v>3</v>
@@ -1938,37 +2121,43 @@
       <c r="M28">
         <v>3</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C29">
         <v>8547224301</v>
       </c>
       <c r="D29" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="E29" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="F29" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="G29" t="s">
+        <v>143</v>
+      </c>
+      <c r="H29" t="s">
+        <v>144</v>
+      </c>
+      <c r="I29">
         <v>16</v>
       </c>
-      <c r="H29" t="s">
-        <v>17</v>
-      </c>
-      <c r="I29">
-        <v>12</v>
-      </c>
       <c r="J29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29">
         <v>4</v>
@@ -1979,37 +2168,43 @@
       <c r="M29">
         <v>4</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="C30">
         <v>9998667888</v>
       </c>
       <c r="D30" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F30" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="G30" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H30" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I30">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K30">
         <v>4</v>
@@ -2020,31 +2215,37 @@
       <c r="M30">
         <v>4</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>43</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="C31">
         <v>6379553392</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E31" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="F31" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="G31" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H31" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I31">
         <v>7</v>
@@ -2061,37 +2262,43 @@
       <c r="M31">
         <v>3</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15">
       <c r="A32" t="s">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C32">
         <v>7877984342</v>
       </c>
       <c r="D32" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="E32" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="F32" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="G32" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H32" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I32">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K32">
         <v>3</v>
@@ -2102,37 +2309,43 @@
       <c r="M32">
         <v>4</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15">
       <c r="A33" t="s">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="C33">
         <v>8369179576</v>
       </c>
       <c r="D33" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="F33" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="G33" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H33" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33">
         <v>1</v>
@@ -2143,31 +2356,37 @@
       <c r="M33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15">
       <c r="A34" t="s">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="B34" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="C34">
         <v>8075327997</v>
       </c>
       <c r="D34" t="s">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="E34" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="F34" t="s">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="G34" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H34" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -2184,31 +2403,37 @@
       <c r="M34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15">
       <c r="A35" t="s">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="B35" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="C35">
         <v>9482712848</v>
       </c>
       <c r="D35" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="F35" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="G35" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H35" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -2225,31 +2450,37 @@
       <c r="M35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15">
       <c r="A36" t="s">
-        <v>113</v>
+        <v>48</v>
       </c>
       <c r="B36" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="C36">
         <v>9500365662</v>
       </c>
       <c r="D36" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="E36" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="F36" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="G36" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H36" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -2266,31 +2497,37 @@
       <c r="M36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N36">
+        <v>0</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15">
       <c r="A37" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="C37">
         <v>9840502912</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="E37" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="F37" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="G37" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H37" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I37">
         <v>8</v>
@@ -2307,31 +2544,37 @@
       <c r="M37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
       <c r="A38" t="s">
-        <v>119</v>
+        <v>50</v>
       </c>
       <c r="B38" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="C38">
         <v>9884198689</v>
       </c>
       <c r="D38" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="E38" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="F38" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="G38" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H38" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I38">
         <v>7</v>
@@ -2348,37 +2591,43 @@
       <c r="M38">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39" t="s">
-        <v>122</v>
+        <v>51</v>
       </c>
       <c r="B39" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="C39">
         <v>7606996818</v>
       </c>
       <c r="D39" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="F39" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="G39" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H39" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I39">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K39">
         <v>4</v>
@@ -2389,31 +2638,37 @@
       <c r="M39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15">
       <c r="A40" t="s">
-        <v>125</v>
+        <v>52</v>
       </c>
       <c r="B40" t="s">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="C40">
         <v>7013522537</v>
       </c>
       <c r="D40" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="E40" t="s">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="F40" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="G40" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H40" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I40">
         <v>2</v>
@@ -2430,31 +2685,37 @@
       <c r="M40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15">
       <c r="A41" t="s">
-        <v>128</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="C41">
         <v>9734187783</v>
       </c>
       <c r="D41" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E41" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="F41" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="G41" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H41" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I41">
         <v>9</v>
@@ -2471,31 +2732,37 @@
       <c r="M41">
         <v>5</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
       <c r="C42">
         <v>9361201097</v>
       </c>
       <c r="D42" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E42" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
       <c r="F42" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G42" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H42" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I42">
         <v>1</v>
@@ -2512,37 +2779,43 @@
       <c r="M42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N42">
+        <v>0</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15">
       <c r="A43" t="s">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>135</v>
+        <v>98</v>
       </c>
       <c r="C43">
         <v>9150943024</v>
       </c>
       <c r="D43" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E43" t="s">
-        <v>135</v>
+        <v>98</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G43" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H43" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="I43">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K43">
         <v>3</v>
@@ -2553,31 +2826,37 @@
       <c r="M43">
         <v>4</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15">
       <c r="A44" t="s">
-        <v>137</v>
+        <v>56</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="C44">
         <v>8637447960</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G44" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H44" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I44">
         <v>8</v>
@@ -2594,13 +2873,19 @@
       <c r="M44">
         <v>2</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15">
       <c r="A45" t="s">
-        <v>140</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="C45">
         <v>9042769165</v>
@@ -2609,16 +2894,16 @@
         <v>142</v>
       </c>
       <c r="E45" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="F45" t="s">
         <v>142</v>
       </c>
       <c r="G45" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H45" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="I45">
         <v>5</v>
@@ -2635,8 +2920,14 @@
       <c r="M45">
         <v>1</v>
       </c>
+      <c r="N45">
+        <v>0</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>